<commit_message>
refactor: restructure P&L analysis and fix data quality issues
Major changes:
- Refactor P&L output to 2 sheets (Daily_Total_PnL, Stock_Total_PnL)
- Update pie chart to show all stocks with ≥5% contribution
- Filter currency assets and problematic stocks at data load level
- Fix alternative returns and graduation analysis to exclude new positions on first day
- Align dual y-axes zero lines in P&L charts
- Add ANALYSIS_SUMMARY.md documentation

Bug fixes:
- Fix graduation chart generation (sheet name mismatch)
- Exclude new positions (Yesterday_Value = 0) from return calculations
- Filter out TCS LI Equity (stock split data issue)
- Skip non-trading days in return calculations

Data updates:
- Update all ETF input data from Bloomberg
- Regenerate ARKF and ARKK analysis outputs
- Remove obsolete ARKG, ARKQ, ARKW, ARKX outputs (to be regenerated)
</commit_message>
<xml_diff>
--- a/output/ARKF/00_Starter_Residual_5_to_7.5pct/ARKF_starter_residual_analysis.xlsx
+++ b/output/ARKF/00_Starter_Residual_5_to_7.5pct/ARKF_starter_residual_analysis.xlsx
@@ -537,10 +537,10 @@
         <v>918.3333333333334</v>
       </c>
       <c r="H2" t="n">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="I2" t="n">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="J2" t="n">
         <v>5</v>
@@ -549,16 +549,16 @@
         <v>2</v>
       </c>
       <c r="L2" t="n">
-        <v>87.03703703703704</v>
+        <v>87.27272727272727</v>
       </c>
       <c r="M2" t="n">
-        <v>80.05555555555556</v>
+        <v>82.40000000000001</v>
       </c>
       <c r="N2" t="n">
-        <v>36</v>
+        <v>10</v>
       </c>
       <c r="O2" t="n">
-        <v>280</v>
+        <v>668.1</v>
       </c>
     </row>
   </sheetData>
@@ -718,7 +718,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I55"/>
+  <dimension ref="A1:I56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -790,7 +790,7 @@
         <v>14.89901692603546</v>
       </c>
       <c r="G2" t="n">
-        <v>6.308591543797745</v>
+        <v>7.358811195222178</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
@@ -823,7 +823,7 @@
         <v>14.89901692603546</v>
       </c>
       <c r="G3" t="n">
-        <v>6.308591543797745</v>
+        <v>7.358811195222178</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
@@ -856,7 +856,7 @@
         <v>14.89901692603546</v>
       </c>
       <c r="G4" t="n">
-        <v>6.308591543797745</v>
+        <v>7.358811195222178</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
@@ -889,7 +889,7 @@
         <v>14.89901692603546</v>
       </c>
       <c r="G5" t="n">
-        <v>6.308591543797745</v>
+        <v>7.358811195222178</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
@@ -922,7 +922,7 @@
         <v>14.89901692603546</v>
       </c>
       <c r="G6" t="n">
-        <v>6.308591543797745</v>
+        <v>7.358811195222178</v>
       </c>
       <c r="H6" t="inlineStr">
         <is>
@@ -955,7 +955,7 @@
         <v>14.89901692603546</v>
       </c>
       <c r="G7" t="n">
-        <v>6.308591543797745</v>
+        <v>7.358811195222178</v>
       </c>
       <c r="H7" t="inlineStr">
         <is>
@@ -988,7 +988,7 @@
         <v>14.89901692603546</v>
       </c>
       <c r="G8" t="n">
-        <v>6.308591543797745</v>
+        <v>7.358811195222178</v>
       </c>
       <c r="H8" t="inlineStr">
         <is>
@@ -1021,7 +1021,7 @@
         <v>14.89901692603546</v>
       </c>
       <c r="G9" t="n">
-        <v>6.308591543797745</v>
+        <v>7.358811195222178</v>
       </c>
       <c r="H9" t="inlineStr">
         <is>
@@ -1054,7 +1054,7 @@
         <v>14.89901692603546</v>
       </c>
       <c r="G10" t="n">
-        <v>6.308591543797745</v>
+        <v>7.358811195222178</v>
       </c>
       <c r="H10" t="inlineStr">
         <is>
@@ -1087,7 +1087,7 @@
         <v>14.89901692603546</v>
       </c>
       <c r="G11" t="n">
-        <v>6.308591543797745</v>
+        <v>7.358811195222178</v>
       </c>
       <c r="H11" t="inlineStr">
         <is>
@@ -1120,7 +1120,7 @@
         <v>14.89901692603546</v>
       </c>
       <c r="G12" t="n">
-        <v>6.308591543797745</v>
+        <v>7.358811195222178</v>
       </c>
       <c r="H12" t="inlineStr">
         <is>
@@ -1153,7 +1153,7 @@
         <v>12.34720565496259</v>
       </c>
       <c r="G13" t="n">
-        <v>6.308591543797745</v>
+        <v>7.358811195222178</v>
       </c>
       <c r="H13" t="inlineStr">
         <is>
@@ -1186,7 +1186,7 @@
         <v>12.34720565496259</v>
       </c>
       <c r="G14" t="n">
-        <v>6.308591543797745</v>
+        <v>7.358811195222178</v>
       </c>
       <c r="H14" t="inlineStr">
         <is>
@@ -1219,7 +1219,7 @@
         <v>10.08446227882257</v>
       </c>
       <c r="G15" t="n">
-        <v>6.308591543797745</v>
+        <v>7.358811195222178</v>
       </c>
       <c r="H15" t="inlineStr">
         <is>
@@ -1252,7 +1252,7 @@
         <v>10.08446227882257</v>
       </c>
       <c r="G16" t="n">
-        <v>6.308591543797745</v>
+        <v>7.358811195222178</v>
       </c>
       <c r="H16" t="inlineStr">
         <is>
@@ -1285,7 +1285,7 @@
         <v>10.08446227882257</v>
       </c>
       <c r="G17" t="n">
-        <v>6.308591543797745</v>
+        <v>7.358811195222178</v>
       </c>
       <c r="H17" t="inlineStr">
         <is>
@@ -1318,7 +1318,7 @@
         <v>10.08446227882257</v>
       </c>
       <c r="G18" t="n">
-        <v>6.308591543797745</v>
+        <v>7.358811195222178</v>
       </c>
       <c r="H18" t="inlineStr">
         <is>
@@ -1351,7 +1351,7 @@
         <v>10.08446227882257</v>
       </c>
       <c r="G19" t="n">
-        <v>6.308591543797745</v>
+        <v>7.358811195222178</v>
       </c>
       <c r="H19" t="inlineStr">
         <is>
@@ -1384,7 +1384,7 @@
         <v>9.597515700974244</v>
       </c>
       <c r="G20" t="n">
-        <v>6.308591543797745</v>
+        <v>7.358811195222178</v>
       </c>
       <c r="H20" t="inlineStr">
         <is>
@@ -1417,7 +1417,7 @@
         <v>7.572908422057561</v>
       </c>
       <c r="G21" t="n">
-        <v>6.308591543797745</v>
+        <v>7.358811195222178</v>
       </c>
       <c r="H21" t="inlineStr">
         <is>
@@ -1447,10 +1447,10 @@
         <v>8.076764546358021</v>
       </c>
       <c r="F22" t="n">
-        <v>6.82225237967744</v>
+        <v>7.377606477370064</v>
       </c>
       <c r="G22" t="n">
-        <v>6.308591543797745</v>
+        <v>7.358811195222178</v>
       </c>
       <c r="H22" t="inlineStr">
         <is>
@@ -1458,7 +1458,7 @@
         </is>
       </c>
       <c r="I22" t="n">
-        <v>25</v>
+        <v>67</v>
       </c>
     </row>
     <row r="23">
@@ -1483,7 +1483,7 @@
         <v>6.9112898248993</v>
       </c>
       <c r="G23" t="n">
-        <v>3.724042079262133</v>
+        <v>3.979064394301959</v>
       </c>
       <c r="H23" t="inlineStr">
         <is>
@@ -1491,7 +1491,7 @@
         </is>
       </c>
       <c r="I23" t="n">
-        <v>65</v>
+        <v>107</v>
       </c>
     </row>
     <row r="24">
@@ -1504,19 +1504,19 @@
         <v>45182</v>
       </c>
       <c r="C24" t="n">
-        <v>100</v>
+        <v>7.579943621481991</v>
       </c>
       <c r="D24" t="n">
         <v>7.299257463036958</v>
       </c>
       <c r="E24" t="n">
-        <v>92.70074253696305</v>
+        <v>0.2806861584450333</v>
       </c>
       <c r="F24" t="n">
         <v>8.032132497172121</v>
       </c>
       <c r="G24" t="n">
-        <v>2.198252955153464</v>
+        <v>1.574645848741667</v>
       </c>
       <c r="H24" t="inlineStr">
         <is>
@@ -1537,19 +1537,19 @@
         <v>45189</v>
       </c>
       <c r="C25" t="n">
-        <v>100</v>
+        <v>7.710923156324315</v>
       </c>
       <c r="D25" t="n">
         <v>7.490065273120071</v>
       </c>
       <c r="E25" t="n">
-        <v>92.50993472687993</v>
+        <v>0.2208578832042436</v>
       </c>
       <c r="F25" t="n">
         <v>8.032132497172121</v>
       </c>
       <c r="G25" t="n">
-        <v>2.198252955153464</v>
+        <v>1.574645848741667</v>
       </c>
       <c r="H25" t="inlineStr">
         <is>
@@ -1570,19 +1570,19 @@
         <v>45259</v>
       </c>
       <c r="C26" t="n">
-        <v>100</v>
+        <v>8.032132497172121</v>
       </c>
       <c r="D26" t="n">
         <v>7.352700754251599</v>
       </c>
       <c r="E26" t="n">
-        <v>92.6472992457484</v>
+        <v>0.6794317429205217</v>
       </c>
       <c r="F26" t="n">
         <v>7.377270929258117</v>
       </c>
       <c r="G26" t="n">
-        <v>2.198252955153464</v>
+        <v>1.574645848741667</v>
       </c>
       <c r="H26" t="inlineStr">
         <is>
@@ -1590,7 +1590,7 @@
         </is>
       </c>
       <c r="I26" t="n">
-        <v>639</v>
+        <v>681</v>
       </c>
     </row>
     <row r="27">
@@ -1615,7 +1615,7 @@
         <v>9.573358807283071</v>
       </c>
       <c r="G27" t="n">
-        <v>7.031976110151669</v>
+        <v>5.963798767672147</v>
       </c>
       <c r="H27" t="inlineStr">
         <is>
@@ -1648,7 +1648,7 @@
         <v>9.573358807283071</v>
       </c>
       <c r="G28" t="n">
-        <v>7.031976110151669</v>
+        <v>5.963798767672147</v>
       </c>
       <c r="H28" t="inlineStr">
         <is>
@@ -1681,7 +1681,7 @@
         <v>7.852974060399701</v>
       </c>
       <c r="G29" t="n">
-        <v>7.031976110151669</v>
+        <v>5.963798767672147</v>
       </c>
       <c r="H29" t="inlineStr">
         <is>
@@ -1711,51 +1711,51 @@
         <v>2.137634824821192</v>
       </c>
       <c r="F30" t="n">
-        <v>7.455585912710889</v>
+        <v>7.784727976919113</v>
       </c>
       <c r="G30" t="n">
-        <v>7.031976110151669</v>
+        <v>5.963798767672147</v>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>Still Residual</t>
+          <t>Recovered to Large</t>
         </is>
       </c>
       <c r="I30" t="n">
-        <v>8</v>
+        <v>19</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>PATH US Equity</t>
+          <t>HOOD US Equity</t>
         </is>
       </c>
       <c r="B31" s="2" t="n">
-        <v>44743</v>
+        <v>45910</v>
       </c>
       <c r="C31" t="n">
-        <v>7.702111336570387</v>
+        <v>9.573358807283071</v>
       </c>
       <c r="D31" t="n">
-        <v>7.333554518124111</v>
+        <v>6.940003306650663</v>
       </c>
       <c r="E31" t="n">
-        <v>0.368556818446276</v>
+        <v>2.633355500632408</v>
       </c>
       <c r="F31" t="n">
-        <v>7.714164468316685</v>
+        <v>6.940003306650663</v>
       </c>
       <c r="G31" t="n">
-        <v>0</v>
+        <v>5.963798767672147</v>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>Recovered to Large</t>
+          <t>Still Residual</t>
         </is>
       </c>
       <c r="I31" t="n">
-        <v>5</v>
+        <v>30</v>
       </c>
     </row>
     <row r="32">
@@ -1765,19 +1765,19 @@
         </is>
       </c>
       <c r="B32" s="2" t="n">
-        <v>44755</v>
+        <v>44743</v>
       </c>
       <c r="C32" t="n">
+        <v>7.702111336570387</v>
+      </c>
+      <c r="D32" t="n">
+        <v>7.333554518124111</v>
+      </c>
+      <c r="E32" t="n">
+        <v>0.368556818446276</v>
+      </c>
+      <c r="F32" t="n">
         <v>7.714164468316685</v>
-      </c>
-      <c r="D32" t="n">
-        <v>7.420455181904349</v>
-      </c>
-      <c r="E32" t="n">
-        <v>0.2937092864123363</v>
-      </c>
-      <c r="F32" t="n">
-        <v>7.566439775688953</v>
       </c>
       <c r="G32" t="n">
         <v>0</v>
@@ -1788,7 +1788,7 @@
         </is>
       </c>
       <c r="I32" t="n">
-        <v>509</v>
+        <v>5</v>
       </c>
     </row>
     <row r="33">
@@ -1798,63 +1798,63 @@
         </is>
       </c>
       <c r="B33" s="2" t="n">
-        <v>45266</v>
+        <v>44755</v>
       </c>
       <c r="C33" t="n">
         <v>7.714164468316685</v>
       </c>
       <c r="D33" t="n">
-        <v>7.296707664620189</v>
+        <v>7.420455181904349</v>
       </c>
       <c r="E33" t="n">
-        <v>0.4174568036964965</v>
+        <v>0.2937092864123363</v>
       </c>
       <c r="F33" t="n">
-        <v>7.296707664620189</v>
+        <v>7.566439775688953</v>
       </c>
       <c r="G33" t="n">
         <v>0</v>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>Dropped</t>
+          <t>Recovered to Large</t>
         </is>
       </c>
       <c r="I33" t="n">
-        <v>533</v>
+        <v>509</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>SHOP CN Equity</t>
+          <t>PATH US Equity</t>
         </is>
       </c>
       <c r="B34" s="2" t="n">
-        <v>44546</v>
+        <v>45266</v>
       </c>
       <c r="C34" t="n">
-        <v>8.103229906452462</v>
+        <v>7.714164468316685</v>
       </c>
       <c r="D34" t="n">
-        <v>7.494864566817361</v>
+        <v>7.296707664620189</v>
       </c>
       <c r="E34" t="n">
-        <v>0.6083653396351014</v>
+        <v>0.4174568036964965</v>
       </c>
       <c r="F34" t="n">
-        <v>52.2282354545503</v>
+        <v>7.296707664620189</v>
       </c>
       <c r="G34" t="n">
-        <v>9.640717166494472</v>
+        <v>0</v>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>Recovered to Large</t>
+          <t>Dropped</t>
         </is>
       </c>
       <c r="I34" t="n">
-        <v>1</v>
+        <v>533</v>
       </c>
     </row>
     <row r="35">
@@ -1864,22 +1864,22 @@
         </is>
       </c>
       <c r="B35" s="2" t="n">
-        <v>44550</v>
+        <v>44546</v>
       </c>
       <c r="C35" t="n">
         <v>8.103229906452462</v>
       </c>
       <c r="D35" t="n">
-        <v>7.435267390802723</v>
+        <v>7.494864566817361</v>
       </c>
       <c r="E35" t="n">
-        <v>0.6679625156497391</v>
+        <v>0.6083653396351014</v>
       </c>
       <c r="F35" t="n">
         <v>52.2282354545503</v>
       </c>
       <c r="G35" t="n">
-        <v>9.640717166494472</v>
+        <v>10.1728501816377</v>
       </c>
       <c r="H35" t="inlineStr">
         <is>
@@ -1887,7 +1887,7 @@
         </is>
       </c>
       <c r="I35" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="36">
@@ -1897,22 +1897,22 @@
         </is>
       </c>
       <c r="B36" s="2" t="n">
-        <v>44566</v>
+        <v>44550</v>
       </c>
       <c r="C36" t="n">
         <v>8.103229906452462</v>
       </c>
       <c r="D36" t="n">
-        <v>7.067708819938829</v>
+        <v>7.435267390802723</v>
       </c>
       <c r="E36" t="n">
-        <v>1.035521086513633</v>
+        <v>0.6679625156497391</v>
       </c>
       <c r="F36" t="n">
         <v>52.2282354545503</v>
       </c>
       <c r="G36" t="n">
-        <v>9.640717166494472</v>
+        <v>10.1728501816377</v>
       </c>
       <c r="H36" t="inlineStr">
         <is>
@@ -1920,7 +1920,7 @@
         </is>
       </c>
       <c r="I36" t="n">
-        <v>14</v>
+        <v>2</v>
       </c>
     </row>
     <row r="37">
@@ -1930,22 +1930,22 @@
         </is>
       </c>
       <c r="B37" s="2" t="n">
-        <v>44585</v>
+        <v>44566</v>
       </c>
       <c r="C37" t="n">
         <v>8.103229906452462</v>
       </c>
       <c r="D37" t="n">
-        <v>7.175629201631434</v>
+        <v>7.067708819938829</v>
       </c>
       <c r="E37" t="n">
-        <v>0.9276007048210282</v>
+        <v>1.035521086513633</v>
       </c>
       <c r="F37" t="n">
         <v>52.2282354545503</v>
       </c>
       <c r="G37" t="n">
-        <v>9.640717166494472</v>
+        <v>10.1728501816377</v>
       </c>
       <c r="H37" t="inlineStr">
         <is>
@@ -1953,7 +1953,7 @@
         </is>
       </c>
       <c r="I37" t="n">
-        <v>1</v>
+        <v>14</v>
       </c>
     </row>
     <row r="38">
@@ -1963,22 +1963,22 @@
         </is>
       </c>
       <c r="B38" s="2" t="n">
-        <v>44587</v>
+        <v>44585</v>
       </c>
       <c r="C38" t="n">
         <v>8.103229906452462</v>
       </c>
       <c r="D38" t="n">
-        <v>7.39699314514213</v>
+        <v>7.175629201631434</v>
       </c>
       <c r="E38" t="n">
-        <v>0.7062367613103326</v>
+        <v>0.9276007048210282</v>
       </c>
       <c r="F38" t="n">
         <v>52.2282354545503</v>
       </c>
       <c r="G38" t="n">
-        <v>9.640717166494472</v>
+        <v>10.1728501816377</v>
       </c>
       <c r="H38" t="inlineStr">
         <is>
@@ -1986,7 +1986,7 @@
         </is>
       </c>
       <c r="I38" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
     </row>
     <row r="39">
@@ -1996,22 +1996,22 @@
         </is>
       </c>
       <c r="B39" s="2" t="n">
-        <v>44609</v>
+        <v>44587</v>
       </c>
       <c r="C39" t="n">
-        <v>8.172284315711268</v>
+        <v>8.103229906452462</v>
       </c>
       <c r="D39" t="n">
-        <v>6.612450900732892</v>
+        <v>7.39699314514213</v>
       </c>
       <c r="E39" t="n">
-        <v>1.559833414978376</v>
+        <v>0.7062367613103326</v>
       </c>
       <c r="F39" t="n">
         <v>52.2282354545503</v>
       </c>
       <c r="G39" t="n">
-        <v>9.640717166494472</v>
+        <v>10.1728501816377</v>
       </c>
       <c r="H39" t="inlineStr">
         <is>
@@ -2019,7 +2019,7 @@
         </is>
       </c>
       <c r="I39" t="n">
-        <v>25</v>
+        <v>6</v>
       </c>
     </row>
     <row r="40">
@@ -2029,22 +2029,22 @@
         </is>
       </c>
       <c r="B40" s="2" t="n">
-        <v>45350</v>
+        <v>44609</v>
       </c>
       <c r="C40" t="n">
+        <v>8.172284315711268</v>
+      </c>
+      <c r="D40" t="n">
+        <v>6.612450900732892</v>
+      </c>
+      <c r="E40" t="n">
+        <v>1.559833414978376</v>
+      </c>
+      <c r="F40" t="n">
         <v>52.2282354545503</v>
       </c>
-      <c r="D40" t="n">
-        <v>7.445757949898097</v>
-      </c>
-      <c r="E40" t="n">
-        <v>44.78247750465221</v>
-      </c>
-      <c r="F40" t="n">
-        <v>11.0722729725144</v>
-      </c>
       <c r="G40" t="n">
-        <v>9.640717166494472</v>
+        <v>10.1728501816377</v>
       </c>
       <c r="H40" t="inlineStr">
         <is>
@@ -2052,7 +2052,7 @@
         </is>
       </c>
       <c r="I40" t="n">
-        <v>70</v>
+        <v>25</v>
       </c>
     </row>
     <row r="41">
@@ -2062,22 +2062,22 @@
         </is>
       </c>
       <c r="B41" s="2" t="n">
-        <v>45421</v>
+        <v>45350</v>
       </c>
       <c r="C41" t="n">
         <v>52.2282354545503</v>
       </c>
       <c r="D41" t="n">
-        <v>6.987147467737483</v>
+        <v>7.445757949898097</v>
       </c>
       <c r="E41" t="n">
-        <v>45.24108798681281</v>
+        <v>44.78247750465221</v>
       </c>
       <c r="F41" t="n">
         <v>11.0722729725144</v>
       </c>
       <c r="G41" t="n">
-        <v>9.640717166494472</v>
+        <v>10.1728501816377</v>
       </c>
       <c r="H41" t="inlineStr">
         <is>
@@ -2085,32 +2085,32 @@
         </is>
       </c>
       <c r="I41" t="n">
-        <v>21</v>
+        <v>70</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>TWLO US Equity</t>
+          <t>SHOP CN Equity</t>
         </is>
       </c>
       <c r="B42" s="2" t="n">
-        <v>44643</v>
+        <v>45421</v>
       </c>
       <c r="C42" t="n">
-        <v>7.521623629374054</v>
+        <v>52.2282354545503</v>
       </c>
       <c r="D42" t="n">
-        <v>7.452096387979089</v>
+        <v>6.987147467737483</v>
       </c>
       <c r="E42" t="n">
-        <v>0.06952724139496524</v>
+        <v>45.24108798681281</v>
       </c>
       <c r="F42" t="n">
-        <v>8.598499657580531</v>
+        <v>11.0722729725144</v>
       </c>
       <c r="G42" t="n">
-        <v>0</v>
+        <v>10.1728501816377</v>
       </c>
       <c r="H42" t="inlineStr">
         <is>
@@ -2118,7 +2118,7 @@
         </is>
       </c>
       <c r="I42" t="n">
-        <v>1</v>
+        <v>21</v>
       </c>
     </row>
     <row r="43">
@@ -2128,16 +2128,16 @@
         </is>
       </c>
       <c r="B43" s="2" t="n">
-        <v>44645</v>
+        <v>44643</v>
       </c>
       <c r="C43" t="n">
         <v>7.521623629374054</v>
       </c>
       <c r="D43" t="n">
-        <v>7.479939829310278</v>
+        <v>7.452096387979089</v>
       </c>
       <c r="E43" t="n">
-        <v>0.04168380006377603</v>
+        <v>0.06952724139496524</v>
       </c>
       <c r="F43" t="n">
         <v>8.598499657580531</v>
@@ -2151,7 +2151,7 @@
         </is>
       </c>
       <c r="I43" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="44">
@@ -2161,16 +2161,16 @@
         </is>
       </c>
       <c r="B44" s="2" t="n">
-        <v>44669</v>
+        <v>44645</v>
       </c>
       <c r="C44" t="n">
-        <v>7.991414907519993</v>
+        <v>7.521623629374054</v>
       </c>
       <c r="D44" t="n">
-        <v>7.424040841933305</v>
+        <v>7.479939829310278</v>
       </c>
       <c r="E44" t="n">
-        <v>0.5673740655866881</v>
+        <v>0.04168380006377603</v>
       </c>
       <c r="F44" t="n">
         <v>8.598499657580531</v>
@@ -2184,7 +2184,7 @@
         </is>
       </c>
       <c r="I44" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
     </row>
     <row r="45">
@@ -2194,16 +2194,16 @@
         </is>
       </c>
       <c r="B45" s="2" t="n">
-        <v>44672</v>
+        <v>44669</v>
       </c>
       <c r="C45" t="n">
         <v>7.991414907519993</v>
       </c>
       <c r="D45" t="n">
-        <v>7.260480646728469</v>
+        <v>7.424040841933305</v>
       </c>
       <c r="E45" t="n">
-        <v>0.7309342607915239</v>
+        <v>0.5673740655866881</v>
       </c>
       <c r="F45" t="n">
         <v>8.598499657580531</v>
@@ -2217,7 +2217,7 @@
         </is>
       </c>
       <c r="I45" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="46">
@@ -2227,16 +2227,16 @@
         </is>
       </c>
       <c r="B46" s="2" t="n">
-        <v>44680</v>
+        <v>44672</v>
       </c>
       <c r="C46" t="n">
         <v>7.991414907519993</v>
       </c>
       <c r="D46" t="n">
-        <v>7.484434271198498</v>
+        <v>7.260480646728469</v>
       </c>
       <c r="E46" t="n">
-        <v>0.5069806363214955</v>
+        <v>0.7309342607915239</v>
       </c>
       <c r="F46" t="n">
         <v>8.598499657580531</v>
@@ -2250,7 +2250,7 @@
         </is>
       </c>
       <c r="I46" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="47">
@@ -2260,19 +2260,19 @@
         </is>
       </c>
       <c r="B47" s="2" t="n">
-        <v>44762</v>
+        <v>44680</v>
       </c>
       <c r="C47" t="n">
+        <v>7.991414907519993</v>
+      </c>
+      <c r="D47" t="n">
+        <v>7.484434271198498</v>
+      </c>
+      <c r="E47" t="n">
+        <v>0.5069806363214955</v>
+      </c>
+      <c r="F47" t="n">
         <v>8.598499657580531</v>
-      </c>
-      <c r="D47" t="n">
-        <v>7.493479453004426</v>
-      </c>
-      <c r="E47" t="n">
-        <v>1.105020204576105</v>
-      </c>
-      <c r="F47" t="n">
-        <v>7.705175226302523</v>
       </c>
       <c r="G47" t="n">
         <v>0</v>
@@ -2283,7 +2283,7 @@
         </is>
       </c>
       <c r="I47" t="n">
-        <v>82</v>
+        <v>7</v>
       </c>
     </row>
     <row r="48">
@@ -2293,16 +2293,16 @@
         </is>
       </c>
       <c r="B48" s="2" t="n">
-        <v>44845</v>
+        <v>44762</v>
       </c>
       <c r="C48" t="n">
         <v>8.598499657580531</v>
       </c>
       <c r="D48" t="n">
-        <v>7.35721846228641</v>
+        <v>7.493479453004426</v>
       </c>
       <c r="E48" t="n">
-        <v>1.241281195294121</v>
+        <v>1.105020204576105</v>
       </c>
       <c r="F48" t="n">
         <v>7.705175226302523</v>
@@ -2316,7 +2316,7 @@
         </is>
       </c>
       <c r="I48" t="n">
-        <v>13</v>
+        <v>82</v>
       </c>
     </row>
     <row r="49">
@@ -2326,63 +2326,63 @@
         </is>
       </c>
       <c r="B49" s="2" t="n">
-        <v>44861</v>
+        <v>44845</v>
       </c>
       <c r="C49" t="n">
         <v>8.598499657580531</v>
       </c>
       <c r="D49" t="n">
-        <v>7.396719284902343</v>
+        <v>7.35721846228641</v>
       </c>
       <c r="E49" t="n">
-        <v>1.201780372678188</v>
+        <v>1.241281195294121</v>
       </c>
       <c r="F49" t="n">
-        <v>7.396719284902343</v>
+        <v>7.705175226302523</v>
       </c>
       <c r="G49" t="n">
         <v>0</v>
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>Dropped</t>
+          <t>Recovered to Large</t>
         </is>
       </c>
       <c r="I49" t="n">
-        <v>559</v>
+        <v>13</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>XYZ US Equity</t>
+          <t>TWLO US Equity</t>
         </is>
       </c>
       <c r="B50" s="2" t="n">
-        <v>44741</v>
+        <v>44861</v>
       </c>
       <c r="C50" t="n">
-        <v>13.84986353941615</v>
+        <v>8.598499657580531</v>
       </c>
       <c r="D50" t="n">
-        <v>5.155769879023193</v>
+        <v>7.396719284902343</v>
       </c>
       <c r="E50" t="n">
-        <v>8.694093660392955</v>
+        <v>1.201780372678188</v>
       </c>
       <c r="F50" t="n">
-        <v>11.93617653036938</v>
+        <v>7.396719284902343</v>
       </c>
       <c r="G50" t="n">
-        <v>3.242466314934898</v>
+        <v>0</v>
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>Recovered to Large</t>
+          <t>Dropped</t>
         </is>
       </c>
       <c r="I50" t="n">
-        <v>1</v>
+        <v>559</v>
       </c>
     </row>
     <row r="51">
@@ -2392,22 +2392,22 @@
         </is>
       </c>
       <c r="B51" s="2" t="n">
-        <v>45180</v>
+        <v>44741</v>
       </c>
       <c r="C51" t="n">
         <v>13.84986353941615</v>
       </c>
       <c r="D51" t="n">
-        <v>7.249709874215991</v>
+        <v>5.155769879023193</v>
       </c>
       <c r="E51" t="n">
-        <v>6.600153665200157</v>
+        <v>8.694093660392955</v>
       </c>
       <c r="F51" t="n">
-        <v>9.08076953158616</v>
+        <v>11.93617653036938</v>
       </c>
       <c r="G51" t="n">
-        <v>3.242466314934898</v>
+        <v>3.017245113947369</v>
       </c>
       <c r="H51" t="inlineStr">
         <is>
@@ -2425,22 +2425,22 @@
         </is>
       </c>
       <c r="B52" s="2" t="n">
-        <v>45189</v>
+        <v>45180</v>
       </c>
       <c r="C52" t="n">
         <v>13.84986353941615</v>
       </c>
       <c r="D52" t="n">
-        <v>7.449946942145933</v>
+        <v>7.249709874215991</v>
       </c>
       <c r="E52" t="n">
-        <v>6.399916597270216</v>
+        <v>6.600153665200157</v>
       </c>
       <c r="F52" t="n">
         <v>9.08076953158616</v>
       </c>
       <c r="G52" t="n">
-        <v>3.242466314934898</v>
+        <v>3.017245113947369</v>
       </c>
       <c r="H52" t="inlineStr">
         <is>
@@ -2448,7 +2448,7 @@
         </is>
       </c>
       <c r="I52" t="n">
-        <v>48</v>
+        <v>1</v>
       </c>
     </row>
     <row r="53">
@@ -2458,22 +2458,22 @@
         </is>
       </c>
       <c r="B53" s="2" t="n">
-        <v>45342</v>
+        <v>45189</v>
       </c>
       <c r="C53" t="n">
         <v>13.84986353941615</v>
       </c>
       <c r="D53" t="n">
-        <v>7.292055474311206</v>
+        <v>7.449946942145933</v>
       </c>
       <c r="E53" t="n">
-        <v>6.557808065104942</v>
+        <v>6.399916597270216</v>
       </c>
       <c r="F53" t="n">
         <v>9.08076953158616</v>
       </c>
       <c r="G53" t="n">
-        <v>3.242466314934898</v>
+        <v>3.017245113947369</v>
       </c>
       <c r="H53" t="inlineStr">
         <is>
@@ -2481,7 +2481,7 @@
         </is>
       </c>
       <c r="I53" t="n">
-        <v>2</v>
+        <v>48</v>
       </c>
     </row>
     <row r="54">
@@ -2491,22 +2491,22 @@
         </is>
       </c>
       <c r="B54" s="2" t="n">
-        <v>45428</v>
+        <v>45342</v>
       </c>
       <c r="C54" t="n">
         <v>13.84986353941615</v>
       </c>
       <c r="D54" t="n">
-        <v>7.489779064343353</v>
+        <v>7.292055474311206</v>
       </c>
       <c r="E54" t="n">
-        <v>6.360084475072795</v>
+        <v>6.557808065104942</v>
       </c>
       <c r="F54" t="n">
-        <v>7.655577850512578</v>
+        <v>9.08076953158616</v>
       </c>
       <c r="G54" t="n">
-        <v>3.242466314934898</v>
+        <v>3.017245113947369</v>
       </c>
       <c r="H54" t="inlineStr">
         <is>
@@ -2514,7 +2514,7 @@
         </is>
       </c>
       <c r="I54" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="55">
@@ -2524,30 +2524,63 @@
         </is>
       </c>
       <c r="B55" s="2" t="n">
-        <v>45435</v>
+        <v>45428</v>
       </c>
       <c r="C55" t="n">
         <v>13.84986353941615</v>
       </c>
       <c r="D55" t="n">
+        <v>7.489779064343353</v>
+      </c>
+      <c r="E55" t="n">
+        <v>6.360084475072795</v>
+      </c>
+      <c r="F55" t="n">
+        <v>7.655577850512578</v>
+      </c>
+      <c r="G55" t="n">
+        <v>3.017245113947369</v>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>Recovered to Large</t>
+        </is>
+      </c>
+      <c r="I55" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>XYZ US Equity</t>
+        </is>
+      </c>
+      <c r="B56" s="2" t="n">
+        <v>45435</v>
+      </c>
+      <c r="C56" t="n">
+        <v>13.84986353941615</v>
+      </c>
+      <c r="D56" t="n">
         <v>7.122518537484352</v>
       </c>
-      <c r="E55" t="n">
+      <c r="E56" t="n">
         <v>6.727345001931797</v>
       </c>
-      <c r="F55" t="n">
+      <c r="F56" t="n">
         <v>7.340981038295119</v>
       </c>
-      <c r="G55" t="n">
-        <v>3.242466314934898</v>
-      </c>
-      <c r="H55" t="inlineStr">
+      <c r="G56" t="n">
+        <v>3.017245113947369</v>
+      </c>
+      <c r="H56" t="inlineStr">
         <is>
           <t>Still Residual</t>
         </is>
       </c>
-      <c r="I55" t="n">
-        <v>463</v>
+      <c r="I56" t="n">
+        <v>505</v>
       </c>
     </row>
   </sheetData>
@@ -2561,7 +2594,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E37"/>
+  <dimension ref="A1:E11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2613,666 +2646,172 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>CAD Curncy</t>
+          <t>BABA US Equity</t>
         </is>
       </c>
       <c r="B3" s="2" t="n">
-        <v>44111</v>
+        <v>44446</v>
       </c>
       <c r="C3" s="2" t="n">
-        <v>44235</v>
+        <v>45923</v>
       </c>
       <c r="D3" t="n">
-        <v>124</v>
+        <v>1477</v>
       </c>
       <c r="E3" t="n">
-        <v>0.2632873394351858</v>
+        <v>0.5474875512866419</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>EUR Curncy</t>
+          <t>META US Equity</t>
         </is>
       </c>
       <c r="B4" s="2" t="n">
-        <v>43521</v>
+        <v>44558</v>
       </c>
       <c r="C4" s="2" t="n">
-        <v>43637</v>
+        <v>45281</v>
       </c>
       <c r="D4" t="n">
-        <v>116</v>
+        <v>723</v>
       </c>
       <c r="E4" t="n">
-        <v>0.001964416139246338</v>
+        <v>0.5092618261890409</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>EUR Curncy</t>
+          <t>NVDA US Equity</t>
         </is>
       </c>
       <c r="B5" s="2" t="n">
-        <v>43641</v>
+        <v>44334</v>
       </c>
       <c r="C5" s="2" t="n">
-        <v>43707</v>
+        <v>44708</v>
       </c>
       <c r="D5" t="n">
-        <v>66</v>
+        <v>374</v>
       </c>
       <c r="E5" t="n">
-        <v>0.3878927770042555</v>
+        <v>0.4042329336493665</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>EUR Curncy</t>
+          <t>PINS US Equity</t>
         </is>
       </c>
       <c r="B6" s="2" t="n">
-        <v>43713</v>
+        <v>44545</v>
       </c>
       <c r="C6" s="2" t="n">
-        <v>43951</v>
+        <v>44952</v>
       </c>
       <c r="D6" t="n">
-        <v>238</v>
+        <v>407</v>
       </c>
       <c r="E6" t="n">
-        <v>0.0001509179929640628</v>
+        <v>0.6843959624037065</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>EUR Curncy</t>
+          <t>PLTR US Equity</t>
         </is>
       </c>
       <c r="B7" s="2" t="n">
-        <v>43986</v>
+        <v>44620</v>
       </c>
       <c r="C7" s="2" t="n">
-        <v>44085</v>
+        <v>45064</v>
       </c>
       <c r="D7" t="n">
-        <v>99</v>
+        <v>444</v>
       </c>
       <c r="E7" t="n">
-        <v>7.238301190557532e-07</v>
+        <v>0.2560260324007131</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>EUR Curncy</t>
+          <t>PYPL US Equity</t>
         </is>
       </c>
       <c r="B8" s="2" t="n">
-        <v>44088</v>
+        <v>44610</v>
       </c>
       <c r="C8" s="2" t="n">
-        <v>44610</v>
+        <v>45436</v>
       </c>
       <c r="D8" t="n">
-        <v>522</v>
+        <v>826</v>
       </c>
       <c r="E8" t="n">
-        <v>0.008251777708662412</v>
+        <v>0.6457146440286845</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>EUR Curncy</t>
+          <t>SE US Equity</t>
         </is>
       </c>
       <c r="B9" s="2" t="n">
-        <v>44614</v>
+        <v>44881</v>
       </c>
       <c r="C9" s="2" t="n">
-        <v>45336</v>
+        <v>45356</v>
       </c>
       <c r="D9" t="n">
-        <v>722</v>
+        <v>475</v>
       </c>
       <c r="E9" t="n">
-        <v>0.1612095762656547</v>
+        <v>0.2505158017269435</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>EUR Curncy</t>
+          <t>SHOP CN Equity</t>
         </is>
       </c>
       <c r="B10" s="2" t="n">
-        <v>45337</v>
+        <v>43900</v>
       </c>
       <c r="C10" s="2" t="n">
-        <v>45385</v>
+        <v>44132</v>
       </c>
       <c r="D10" t="n">
-        <v>48</v>
+        <v>232</v>
       </c>
       <c r="E10" t="n">
-        <v>-0.0001897852011505419</v>
+        <v>0.4834538818653537</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>HKD Curncy</t>
+          <t>TWTR US Equity</t>
         </is>
       </c>
       <c r="B11" s="2" t="n">
-        <v>44032</v>
+        <v>43773</v>
       </c>
       <c r="C11" s="2" t="n">
-        <v>44172</v>
+        <v>44531</v>
       </c>
       <c r="D11" t="n">
-        <v>140</v>
+        <v>758</v>
       </c>
       <c r="E11" t="n">
-        <v>0.06757609380609853</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>HKD Curncy</t>
-        </is>
-      </c>
-      <c r="B12" s="2" t="n">
-        <v>44372</v>
-      </c>
-      <c r="C12" s="2" t="n">
-        <v>44442</v>
-      </c>
-      <c r="D12" t="n">
-        <v>70</v>
-      </c>
-      <c r="E12" t="n">
-        <v>0.2130721935694165</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>HKD Curncy</t>
-        </is>
-      </c>
-      <c r="B13" s="2" t="n">
-        <v>44446</v>
-      </c>
-      <c r="C13" s="2" t="n">
-        <v>45385</v>
-      </c>
-      <c r="D13" t="n">
-        <v>939</v>
-      </c>
-      <c r="E13" t="n">
-        <v>-5.06221859042014e-07</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>JPY Curncy</t>
-        </is>
-      </c>
-      <c r="B14" s="2" t="n">
-        <v>43675</v>
-      </c>
-      <c r="C14" s="2" t="n">
-        <v>43810</v>
-      </c>
-      <c r="D14" t="n">
-        <v>135</v>
-      </c>
-      <c r="E14" t="n">
-        <v>0.0142690742599815</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>JPY Curncy</t>
-        </is>
-      </c>
-      <c r="B15" s="2" t="n">
-        <v>43811</v>
-      </c>
-      <c r="C15" s="2" t="n">
-        <v>43894</v>
-      </c>
-      <c r="D15" t="n">
-        <v>83</v>
-      </c>
-      <c r="E15" t="n">
-        <v>1.011516593765187</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>JPY Curncy</t>
-        </is>
-      </c>
-      <c r="B16" s="2" t="n">
-        <v>43906</v>
-      </c>
-      <c r="C16" s="2" t="n">
-        <v>43971</v>
-      </c>
-      <c r="D16" t="n">
-        <v>65</v>
-      </c>
-      <c r="E16" t="n">
-        <v>0.09051575473033632</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>JPY Curncy</t>
-        </is>
-      </c>
-      <c r="B17" s="2" t="n">
-        <v>43991</v>
-      </c>
-      <c r="C17" s="2" t="n">
-        <v>44025</v>
-      </c>
-      <c r="D17" t="n">
-        <v>34</v>
-      </c>
-      <c r="E17" t="n">
-        <v>0.05187143232492531</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>JPY Curncy</t>
-        </is>
-      </c>
-      <c r="B18" s="2" t="n">
-        <v>44026</v>
-      </c>
-      <c r="C18" s="2" t="n">
-        <v>44067</v>
-      </c>
-      <c r="D18" t="n">
-        <v>41</v>
-      </c>
-      <c r="E18" t="n">
-        <v>0.07743346053086182</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>JPY Curncy</t>
-        </is>
-      </c>
-      <c r="B19" s="2" t="n">
-        <v>44225</v>
-      </c>
-      <c r="C19" s="2" t="n">
-        <v>44266</v>
-      </c>
-      <c r="D19" t="n">
-        <v>41</v>
-      </c>
-      <c r="E19" t="n">
-        <v>0.01131133997354291</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>JPY Curncy</t>
-        </is>
-      </c>
-      <c r="B20" s="2" t="n">
-        <v>44298</v>
-      </c>
-      <c r="C20" s="2" t="n">
-        <v>44342</v>
-      </c>
-      <c r="D20" t="n">
-        <v>44</v>
-      </c>
-      <c r="E20" t="n">
-        <v>0.1330329822073394</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>JPY Curncy</t>
-        </is>
-      </c>
-      <c r="B21" s="2" t="n">
-        <v>44364</v>
-      </c>
-      <c r="C21" s="2" t="n">
-        <v>44610</v>
-      </c>
-      <c r="D21" t="n">
-        <v>246</v>
-      </c>
-      <c r="E21" t="n">
-        <v>0.002443742261310396</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>JPY Curncy</t>
-        </is>
-      </c>
-      <c r="B22" s="2" t="n">
-        <v>44630</v>
-      </c>
-      <c r="C22" s="2" t="n">
-        <v>44690</v>
-      </c>
-      <c r="D22" t="n">
-        <v>60</v>
-      </c>
-      <c r="E22" t="n">
-        <v>0.003012984095514021</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>JPY Curncy</t>
-        </is>
-      </c>
-      <c r="B23" s="2" t="n">
-        <v>44728</v>
-      </c>
-      <c r="C23" s="2" t="n">
-        <v>44778</v>
-      </c>
-      <c r="D23" t="n">
-        <v>50</v>
-      </c>
-      <c r="E23" t="n">
-        <v>0.001416672609090148</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>JPY Curncy</t>
-        </is>
-      </c>
-      <c r="B24" s="2" t="n">
-        <v>44781</v>
-      </c>
-      <c r="C24" s="2" t="n">
-        <v>44957</v>
-      </c>
-      <c r="D24" t="n">
-        <v>176</v>
-      </c>
-      <c r="E24" t="n">
-        <v>0.008081244977611568</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>JPY Curncy</t>
-        </is>
-      </c>
-      <c r="B25" s="2" t="n">
-        <v>44958</v>
-      </c>
-      <c r="C25" s="2" t="n">
-        <v>45079</v>
-      </c>
-      <c r="D25" t="n">
-        <v>121</v>
-      </c>
-      <c r="E25" t="n">
-        <v>0.01569686210095401</v>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>JPY Curncy</t>
-        </is>
-      </c>
-      <c r="B26" s="2" t="n">
-        <v>45082</v>
-      </c>
-      <c r="C26" s="2" t="n">
-        <v>45282</v>
-      </c>
-      <c r="D26" t="n">
-        <v>200</v>
-      </c>
-      <c r="E26" t="n">
-        <v>0.2239422313308192</v>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>JPY Curncy</t>
-        </is>
-      </c>
-      <c r="B27" s="2" t="n">
-        <v>45286</v>
-      </c>
-      <c r="C27" s="2" t="n">
-        <v>45357</v>
-      </c>
-      <c r="D27" t="n">
-        <v>71</v>
-      </c>
-      <c r="E27" t="n">
-        <v>0.5111178541361689</v>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>META US Equity</t>
-        </is>
-      </c>
-      <c r="B28" s="2" t="n">
-        <v>44558</v>
-      </c>
-      <c r="C28" s="2" t="n">
-        <v>45281</v>
-      </c>
-      <c r="D28" t="n">
-        <v>723</v>
-      </c>
-      <c r="E28" t="n">
-        <v>0.5092618261890409</v>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>NVDA US Equity</t>
-        </is>
-      </c>
-      <c r="B29" s="2" t="n">
-        <v>44334</v>
-      </c>
-      <c r="C29" s="2" t="n">
-        <v>44708</v>
-      </c>
-      <c r="D29" t="n">
-        <v>374</v>
-      </c>
-      <c r="E29" t="n">
-        <v>0.4042329336493665</v>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>PINS US Equity</t>
-        </is>
-      </c>
-      <c r="B30" s="2" t="n">
-        <v>44545</v>
-      </c>
-      <c r="C30" s="2" t="n">
-        <v>44952</v>
-      </c>
-      <c r="D30" t="n">
-        <v>407</v>
-      </c>
-      <c r="E30" t="n">
-        <v>0.6843959624037065</v>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>PLTR US Equity</t>
-        </is>
-      </c>
-      <c r="B31" s="2" t="n">
-        <v>44620</v>
-      </c>
-      <c r="C31" s="2" t="n">
-        <v>45064</v>
-      </c>
-      <c r="D31" t="n">
-        <v>444</v>
-      </c>
-      <c r="E31" t="n">
-        <v>0.2560260324007131</v>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>PYPL US Equity</t>
-        </is>
-      </c>
-      <c r="B32" s="2" t="n">
-        <v>44610</v>
-      </c>
-      <c r="C32" s="2" t="n">
-        <v>45436</v>
-      </c>
-      <c r="D32" t="n">
-        <v>826</v>
-      </c>
-      <c r="E32" t="n">
-        <v>0.6457146440286845</v>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>SE US Equity</t>
-        </is>
-      </c>
-      <c r="B33" s="2" t="n">
-        <v>44881</v>
-      </c>
-      <c r="C33" s="2" t="n">
-        <v>45356</v>
-      </c>
-      <c r="D33" t="n">
-        <v>475</v>
-      </c>
-      <c r="E33" t="n">
-        <v>0.2505158017269435</v>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>SHOP CN Equity</t>
-        </is>
-      </c>
-      <c r="B34" s="2" t="n">
-        <v>43900</v>
-      </c>
-      <c r="C34" s="2" t="n">
-        <v>44132</v>
-      </c>
-      <c r="D34" t="n">
-        <v>232</v>
-      </c>
-      <c r="E34" t="n">
-        <v>0.4834538818653537</v>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>TWTR US Equity</t>
-        </is>
-      </c>
-      <c r="B35" s="2" t="n">
-        <v>43773</v>
-      </c>
-      <c r="C35" s="2" t="n">
-        <v>44531</v>
-      </c>
-      <c r="D35" t="n">
-        <v>758</v>
-      </c>
-      <c r="E35" t="n">
         <v>0.5063608440363557</v>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t>ZAR Curncy</t>
-        </is>
-      </c>
-      <c r="B36" s="2" t="n">
-        <v>44959</v>
-      </c>
-      <c r="C36" s="2" t="n">
-        <v>45215</v>
-      </c>
-      <c r="D36" t="n">
-        <v>256</v>
-      </c>
-      <c r="E36" t="n">
-        <v>0.02232509365285203</v>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t>ZAR Curncy</t>
-        </is>
-      </c>
-      <c r="B37" s="2" t="n">
-        <v>45216</v>
-      </c>
-      <c r="C37" s="2" t="n">
-        <v>45385</v>
-      </c>
-      <c r="D37" t="n">
-        <v>169</v>
-      </c>
-      <c r="E37" t="n">
-        <v>-0.0003329798795747985</v>
       </c>
     </row>
   </sheetData>

</xml_diff>